<commit_message>
Update: __pycache__/main.cpython-314.pyc, app.py and 2 others
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -425,70 +425,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Team ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Team Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Message</t>
+          <t>Candidate role</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Candidate's Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate's Email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate's Mobile</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate's Gender</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate's Location</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>User type</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Email_Status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Test User 1</t>
+          <t>UUS866X4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>919876543210</t>
+          <t>nyash</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hello! This is a test message with a community link: https://chat.whatsapp.com/xyz</t>
+          <t>Team Member</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Test Candidate</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>+919876543210</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>College Students</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Test User 2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>919876543211</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Hi! Join our new community: https://chat.whatsapp.com/abc</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>